<commit_message>
feat: altera lógica de exportação dos relatórios de centro de custo
Atualiza o fluxo de exportação dos relatórios de centro de custo para acompanhar as mudanças introduzidas na nova versão do sistema Protheus
</commit_message>
<xml_diff>
--- a/log/log_automacao.xlsx
+++ b/log/log_automacao.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$160</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H85"/>
+  <dimension ref="A1:H160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3888,8 +3888,3008 @@
         <v>77.8</v>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:33:54</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:34:14</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao escolher a opção genericos</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="n">
+        <v>20.3</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:38:57</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:41:13</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="n">
+        <v>136.1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:41:18</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:43:44</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="n">
+        <v>145.8</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:43:49</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:46:09</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="n">
+        <v>139.5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:46:14</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:48:54</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="n">
+        <v>160.1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:49:00</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:51:20</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="n">
+        <v>140.8</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:51:26</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:53:43</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="n">
+        <v>137.7</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:53:49</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:56:05</t>
+        </is>
+      </c>
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="n">
+        <v>136.1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:56:10</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:58:26</t>
+        </is>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="n">
+        <v>135.7</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:58:31</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:00:45</t>
+        </is>
+      </c>
+      <c r="C95" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="n">
+        <v>134.2</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:00:50</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:03:08</t>
+        </is>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="n">
+        <v>137.8</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:03:13</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:05:28</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="n">
+        <v>134.8</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:05:33</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:07:50</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="n">
+        <v>136.4</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:07:55</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:10:10</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="n">
+        <v>134.7</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:10:15</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:12:30</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="n">
+        <v>134.8</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:12:35</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>03/06/2026 15:14:54</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="n">
+        <v>139.6</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>06/07/2026 12:01:02</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>06/07/2026 12:04:23</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F102" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao mover/renomear o arquivo CSV</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="n">
+        <v>200.9</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>06/07/2026 12:04:28</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>06/07/2026 12:07:09</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F103" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao mover/renomear o arquivo CSV</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="n">
+        <v>160.6</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>06/07/2026 12:07:14</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>06/07/2026 12:08:59</t>
+        </is>
+      </c>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F104" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G104" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção operador igual a</t>
+        </is>
+      </c>
+      <c r="H104" s="4" t="n">
+        <v>105.3</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 08:44:13</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 08:46:33</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="n">
+        <v>139.9</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 08:46:38</t>
+        </is>
+      </c>
+      <c r="B106" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 08:48:50</t>
+        </is>
+      </c>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F106" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G106" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao selecionar o tipo ponto e virgula</t>
+        </is>
+      </c>
+      <c r="H106" s="4" t="n">
+        <v>132.5</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 08:55:26</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 08:57:43</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 08:57:48</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:00:05</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G108" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H108" s="2" t="n">
+        <v>137.3</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:00:10</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:02:33</t>
+        </is>
+      </c>
+      <c r="C109" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E109" s="2" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G109" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H109" s="2" t="n">
+        <v>142.1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:02:38</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:05:20</t>
+        </is>
+      </c>
+      <c r="C110" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:05:25</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:07:43</t>
+        </is>
+      </c>
+      <c r="C111" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E111" s="2" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G111" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H111" s="2" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:07:48</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:10:08</t>
+        </is>
+      </c>
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="n">
+        <v>139.4</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:10:13</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:12:28</t>
+        </is>
+      </c>
+      <c r="C113" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="n">
+        <v>135.1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:12:33</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:14:48</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="n">
+        <v>135.1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:14:54</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:17:10</t>
+        </is>
+      </c>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="n">
+        <v>136.1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:17:15</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:19:00</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F116" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G116" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção operador igual a</t>
+        </is>
+      </c>
+      <c r="H116" s="4" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:46:48</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:49:04</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:49:09</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:51:29</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="n">
+        <v>139.8</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:51:34</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:53:52</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="n">
+        <v>137.8</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:53:57</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:57:01</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:57:07</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:59:24</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="n">
+        <v>137.2</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 09:59:29</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:01:47</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="n">
+        <v>138.3</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:01:53</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:04:08</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="n">
+        <v>135.5</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:04:13</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:06:29</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="n">
+        <v>135.5</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:06:34</t>
+        </is>
+      </c>
+      <c r="B125" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:08:47</t>
+        </is>
+      </c>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E125" s="4" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F125" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G125" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao selecionar o tipo ponto e virgula</t>
+        </is>
+      </c>
+      <c r="H125" s="4" t="n">
+        <v>132.7</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:46:33</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:48:48</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>134.8</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:48:53</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:51:11</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>137.1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:51:16</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:53:30</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="n">
+        <v>134.3</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:53:35</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:55:54</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:56:00</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:58:14</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G130" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H130" s="2" t="n">
+        <v>134.2</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 10:58:19</t>
+        </is>
+      </c>
+      <c r="B131" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 11:00:35</t>
+        </is>
+      </c>
+      <c r="C131" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G131" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H131" s="2" t="n">
+        <v>136.2</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 11:00:41</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 11:02:46</t>
+        </is>
+      </c>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F132" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G132" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao selecionar a caixa do filtro criado</t>
+        </is>
+      </c>
+      <c r="H132" s="4" t="n">
+        <v>125.1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 11:05:02</t>
+        </is>
+      </c>
+      <c r="B133" s="2" t="inlineStr">
+        <is>
+          <t>08/07/2026 11:07:21</t>
+        </is>
+      </c>
+      <c r="C133" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G133" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H133" s="2" t="n">
+        <v>139.4</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 11:11:31</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>08/07/2026 11:12:24</t>
+        </is>
+      </c>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>30/06/2026</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F134" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G134" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar no menu Planilha</t>
+        </is>
+      </c>
+      <c r="H134" s="4" t="n">
+        <v>52.4</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:35:02</t>
+        </is>
+      </c>
+      <c r="B135" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:37:17</t>
+        </is>
+      </c>
+      <c r="C135" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F135" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G135" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H135" s="2" t="n">
+        <v>134.8</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:37:22</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:39:38</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G136" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="n">
+        <v>135.8</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:39:43</t>
+        </is>
+      </c>
+      <c r="B137" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:42:02</t>
+        </is>
+      </c>
+      <c r="C137" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G137" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H137" s="2" t="n">
+        <v>138.8</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:42:07</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:44:44</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F138" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G138" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="n">
+        <v>156.6</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:44:49</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:47:08</t>
+        </is>
+      </c>
+      <c r="C139" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G139" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H139" s="2" t="n">
+        <v>139.4</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:47:14</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:48:59</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F140" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G140" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção operador igual a</t>
+        </is>
+      </c>
+      <c r="H140" s="4" t="n">
+        <v>105.2</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:55:42</t>
+        </is>
+      </c>
+      <c r="B141" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:58:00</t>
+        </is>
+      </c>
+      <c r="C141" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="n">
+        <v>137.5</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 09:58:05</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:00:19</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G142" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="n">
+        <v>134.5</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:00:24</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:02:39</t>
+        </is>
+      </c>
+      <c r="C143" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F143" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:02:45</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:05:00</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="n">
+        <v>135.2</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:05:05</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:07:25</t>
+        </is>
+      </c>
+      <c r="C145" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E145" s="2" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G145" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H145" s="2" t="n">
+        <v>140.1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:07:30</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:09:47</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G146" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="n">
+        <v>136.4</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:09:52</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:12:07</t>
+        </is>
+      </c>
+      <c r="C147" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E147" s="2" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G147" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H147" s="2" t="n">
+        <v>135.4</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:12:12</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:14:29</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="n">
+        <v>136.7</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:14:34</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:16:50</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="n">
+        <v>135.6</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="4" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:16:55</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:18:38</t>
+        </is>
+      </c>
+      <c r="C150" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E150" s="4" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F150" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G150" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção data</t>
+        </is>
+      </c>
+      <c r="H150" s="4" t="n">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:29:47</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:32:06</t>
+        </is>
+      </c>
+      <c r="C151" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G151" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H151" s="2" t="n">
+        <v>138.7</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:32:11</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026 10:34:25</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>01010041</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G152" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="4" t="inlineStr">
+        <is>
+          <t>11/08/2026 11:42:03</t>
+        </is>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>11/08/2026 11:42:55</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D153" s="4" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G153" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar no menu Planilha</t>
+        </is>
+      </c>
+      <c r="H153" s="4" t="n">
+        <v>52.4</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:04:45</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:05:02</t>
+        </is>
+      </c>
+      <c r="C154" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F154" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G154" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao acessar a opção Smart View</t>
+        </is>
+      </c>
+      <c r="H154" s="4" t="n">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:06:43</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:07:36</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G155" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção selecionada para exportar planilha</t>
+        </is>
+      </c>
+      <c r="H155" s="4" t="n">
+        <v>53.1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:16:58</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:17:53</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F156" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G156" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção selecionada para exportar planilha</t>
+        </is>
+      </c>
+      <c r="H156" s="4" t="n">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:27:19</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:28:24</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G157" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao selecionar o tipo CSV</t>
+        </is>
+      </c>
+      <c r="H157" s="4" t="n">
+        <v>65.3</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:42:34</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 14:43:39</t>
+        </is>
+      </c>
+      <c r="C158" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F158" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G158" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao selecionar o tipo CSV</t>
+        </is>
+      </c>
+      <c r="H158" s="4" t="n">
+        <v>65.3</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 16:20:38</t>
+        </is>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 16:21:33</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D159" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E159" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G159" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na opção selecionada para exportar planilha</t>
+        </is>
+      </c>
+      <c r="H159" s="4" t="n">
+        <v>54.9</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 16:28:38</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>01/09/2026 16:30:36</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F160" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar no botão Salvar Arquivo na janela de salvar</t>
+        </is>
+      </c>
+      <c r="H160" s="4" t="n">
+        <v>118.8</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H85"/>
+  <autoFilter ref="A1:H160"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: adiciona margem para aguardar o download do relatório de centro de custo e pausa ao digitar as competências no relatório de consumo
</commit_message>
<xml_diff>
--- a/log/log_automacao.xlsx
+++ b/log/log_automacao.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Log'!$A$1:$H$185</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -473,7 +473,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6888,8 +6888,1008 @@
         <v>118.8</v>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" s="4" t="inlineStr">
+        <is>
+          <t>02/09/2026 08:44:11</t>
+        </is>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>02/09/2026 08:45:06</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D161" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G161" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar no botão Confirmar Exportação</t>
+        </is>
+      </c>
+      <c r="H161" s="4" t="n">
+        <v>54.7</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>02/09/2026 08:54:39</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>02/09/2026 08:55:34</t>
+        </is>
+      </c>
+      <c r="C162" s="4" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F162" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G162" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar no botão Confirmar Exportação</t>
+        </is>
+      </c>
+      <c r="H162" s="4" t="n">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:18:48</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:20:22</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010035_31-08-2026.csv</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="n">
+        <v>93.90000000000001</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:20:22</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:21:45</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G164" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010037_31-08-2026.csv</t>
+        </is>
+      </c>
+      <c r="H164" s="2" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:21:45</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:23:04</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010038_31-08-2026.csv</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="n">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:23:05</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:24:26</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F166" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010039_31-08-2026.csv</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="n">
+        <v>81.8</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:24:27</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:25:47</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010048_31-08-2026.csv</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="n">
+        <v>80.3</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:25:47</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:27:08</t>
+        </is>
+      </c>
+      <c r="C168" s="2" t="inlineStr">
+        <is>
+          <t>Centro de Custo</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E168" s="2" t="inlineStr">
+        <is>
+          <t>01010041</t>
+        </is>
+      </c>
+      <c r="F168" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G168" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo gerado e renomeado: CC_01010041_31-08-2026.csv</t>
+        </is>
+      </c>
+      <c r="H168" s="2" t="n">
+        <v>80.8</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:30:11</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:31:18</t>
+        </is>
+      </c>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E169" s="4" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>❌ Erro</t>
+        </is>
+      </c>
+      <c r="G169" s="4" t="inlineStr">
+        <is>
+          <t>Erro ao clicar na caixa de texto</t>
+        </is>
+      </c>
+      <c r="H169" s="4" t="n">
+        <v>66.3</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:36:38</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:38:52</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>01010009</t>
+        </is>
+      </c>
+      <c r="F170" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="n">
+        <v>134.1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:38:57</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:41:13</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>01010010</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="n">
+        <v>135.9</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:41:18</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:43:43</t>
+        </is>
+      </c>
+      <c r="C172" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E172" s="2" t="inlineStr">
+        <is>
+          <t>01010034</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G172" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H172" s="2" t="n">
+        <v>144.7</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:43:48</t>
+        </is>
+      </c>
+      <c r="B173" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:46:43</t>
+        </is>
+      </c>
+      <c r="C173" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E173" s="2" t="inlineStr">
+        <is>
+          <t>01010040</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G173" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H173" s="2" t="n">
+        <v>175.2</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:46:48</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:49:04</t>
+        </is>
+      </c>
+      <c r="C174" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E174" s="2" t="inlineStr">
+        <is>
+          <t>01010044</t>
+        </is>
+      </c>
+      <c r="F174" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G174" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H174" s="2" t="n">
+        <v>135.9</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:49:09</t>
+        </is>
+      </c>
+      <c r="B175" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:51:23</t>
+        </is>
+      </c>
+      <c r="C175" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E175" s="2" t="inlineStr">
+        <is>
+          <t>01010057</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G175" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H175" s="2" t="n">
+        <v>133.4</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:51:28</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:53:41</t>
+        </is>
+      </c>
+      <c r="C176" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>01010011</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:53:46</t>
+        </is>
+      </c>
+      <c r="B177" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:56:03</t>
+        </is>
+      </c>
+      <c r="C177" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>01010024</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="n">
+        <v>136.5</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:56:08</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:58:22</t>
+        </is>
+      </c>
+      <c r="C178" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>01010027</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="n">
+        <v>133.8</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 09:58:27</t>
+        </is>
+      </c>
+      <c r="B179" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:02:44</t>
+        </is>
+      </c>
+      <c r="C179" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>01010028</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="n">
+        <v>256.9</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:02:49</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:05:05</t>
+        </is>
+      </c>
+      <c r="C180" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>01010035</t>
+        </is>
+      </c>
+      <c r="F180" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:05:10</t>
+        </is>
+      </c>
+      <c r="B181" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:07:25</t>
+        </is>
+      </c>
+      <c r="C181" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E181" s="2" t="inlineStr">
+        <is>
+          <t>01010037</t>
+        </is>
+      </c>
+      <c r="F181" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G181" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H181" s="2" t="n">
+        <v>134.7</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:07:30</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:09:47</t>
+        </is>
+      </c>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>01010038</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="n">
+        <v>136.8</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:09:52</t>
+        </is>
+      </c>
+      <c r="B183" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:12:07</t>
+        </is>
+      </c>
+      <c r="C183" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E183" s="2" t="inlineStr">
+        <is>
+          <t>01010039</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G183" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H183" s="2" t="n">
+        <v>134.6</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:12:12</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:14:33</t>
+        </is>
+      </c>
+      <c r="C184" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>01010048</t>
+        </is>
+      </c>
+      <c r="F184" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G184" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H184" s="2" t="n">
+        <v>140.7</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:14:38</t>
+        </is>
+      </c>
+      <c r="B185" s="2" t="inlineStr">
+        <is>
+          <t>02/09/2026 10:16:54</t>
+        </is>
+      </c>
+      <c r="C185" s="2" t="inlineStr">
+        <is>
+          <t>Consumo</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
+      <c r="E185" s="2" t="inlineStr">
+        <is>
+          <t>01010041</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>✅ Sucesso</t>
+        </is>
+      </c>
+      <c r="G185" s="2" t="inlineStr">
+        <is>
+          <t>Arquivo exportado e movido com sucesso</t>
+        </is>
+      </c>
+      <c r="H185" s="2" t="n">
+        <v>136.7</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H160"/>
+  <autoFilter ref="A1:H185"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>